<commit_message>
Clarify Garden POC roadmap proof
</commit_message>
<xml_diff>
--- a/sheets/jarvis_roadmap.xlsx
+++ b/sheets/jarvis_roadmap.xlsx
@@ -805,7 +805,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Near-term priority: prove one v0 protocol loop end to end: protocol lock, schemas, version and capability negotiation, adapter contract, first host POC mapping, portable export, and conformance fixtures. Keep scope narrow: protocol records first, one product host plus one CLI/existing-agent wrapper, evidence and learning captured during work.</t>
+          <t>Near-term priority: prove one v0 protocol loop end to end: protocol lock, schemas, version and capability negotiation, adapter contract, Garden POC mapping, portable export, and conformance fixtures. Garden POC is the product proof before main Garden adopts the protocol. Keep scope narrow: protocol records first, Garden POC plus one CLI/existing-agent wrapper, evidence and learning captured during work.</t>
         </is>
       </c>
       <c r="B4" s="30" t="n"/>
@@ -875,7 +875,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Host POC + demo</t>
+          <t>Garden POC + demo</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -926,15 +926,15 @@
       </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
-          <t>- choose first product host proof
+          <t>- choose Garden POC as the first product proof
 - choose one CLI/external-agent wrapper
-- define host-private fields that stay out of export
+- define Garden-private fields that stay out of export
 - define demo success path</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
         <is>
-          <t>Protocol lock is the source for schema work, first host and wrapper targets are named, and no new runtime/product assumptions enter Jarvis.</t>
+          <t>Protocol lock is the source for schema work, Garden POC and wrapper targets are named, and no new runtime/product assumptions enter Jarvis.</t>
         </is>
       </c>
     </row>
@@ -980,8 +980,8 @@
       </c>
       <c r="G8" s="25" t="inlineStr">
         <is>
-          <t>- create first host mapping table
-- define host WorkSession flow
+          <t>- create Garden POC mapping table
+- define Garden WorkSession flow
 - define Request inbox behavior
 - define Review and Takeover capture points</t>
         </is>
@@ -1021,7 +1021,7 @@
           <t>- build golden-path fixtures
 - build failing fixtures
 - validate status transitions
-- validate export does not require host-private fields</t>
+- validate export does not require Garden-private fields</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
-          <t>- run host POC mapping against schemas
+          <t>- run Garden POC mapping against schemas
 - generate sample WorkSession export
 - show evidence and learning records
 - document host-only assumptions separately</t>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="C10" s="25" t="inlineStr">
         <is>
-          <t>Prove Jarvis with the first host and one existing-agent wrapper.</t>
+          <t>Prove Jarvis with Garden POC and one existing-agent wrapper.</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>- demonstrate host POC flow
+          <t>- demonstrate Garden POC flow
 - export EvidenceManifest
 - export LearningRecord
 - show human, agent, and pair learning
@@ -1144,14 +1144,14 @@
       <c r="G11" s="22" t="inlineStr">
         <is>
           <t>- publish final demo URL
-- package host POC evidence
+- package Garden POC evidence
 - prepare team walkthrough
 - collect review notes into next-cycle issues</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
         <is>
-          <t>Jarvis has a v0.1 alpha package of protocol docs, schemas, examples, conformance fixtures, one host proof, and one existing-agent wrapper proof.</t>
+          <t>Jarvis has a v0.1 alpha package of protocol docs, schemas, examples, conformance fixtures, Garden POC proof, and one existing-agent wrapper proof.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G12" s="25" t="inlineStr">
         <is>
-          <t>- additional host proofs
+          <t>- additional product proofs
 - public demo refresh
 - team onboarding sheet
 - protocol review sessions</t>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
-          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and host proof evidence, not by adding features from vibes.</t>
+          <t>Expansion is justified by valid exports, conformance failures, adapter pain, and Garden POC evidence, not by adding features from vibes.</t>
         </is>
       </c>
     </row>

</xml_diff>